<commit_message>
Dev Notes and Sprint Planning Updates
</commit_message>
<xml_diff>
--- a/Business Analysis/checkupp_sprint_plan_2026.xlsx
+++ b/Business Analysis/checkupp_sprint_plan_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\CheckUpp\Business Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5CB78D0-50AC-4087-955E-59A9E659A7A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA2C8B7-F614-444B-8762-C8F096F11AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10907,11 +10907,11 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" customWidth="1"/>
-    <col min="3" max="3" width="7.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.109375" customWidth="1"/>
     <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="99.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="99.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
@@ -10958,7 +10958,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A2" s="15">
         <v>1</v>
       </c>
@@ -11168,7 +11168,7 @@
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
     </row>
-    <row r="8" spans="1:12" ht="99" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A8" s="15">
         <v>7</v>
       </c>

</xml_diff>